<commit_message>
docs: ROI model v4 (one branch pilot, regulator stress, local LLM cost fix)
</commit_message>
<xml_diff>
--- a/docs/roi_model_en.xlsx
+++ b/docs/roi_model_en.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Sample check" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Deck summary" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="395">
   <si>
     <t xml:space="preserve">MAQSAD ROI model: assumptions and inputs</t>
   </si>
@@ -222,10 +222,10 @@
     <t xml:space="preserve">Pilot hours: Backend/Frontend</t>
   </si>
   <si>
-    <t xml:space="preserve">Taxmin: team plan (Oybek, 11 Oct; confirm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One-time: on-prem installation and app work. Base ~340 h (his table sums to 344) = month 1: 168 (install on bank server, bank data adapter, local LLM with GPU, SSO/roles, audit to bank DB, historical test run), month 2: 96 (support, officer-feedback changes, training, monitoring), month 3: 80 (result report, documents). Pessimistic ~520 = complex data connection, many security requirements, GPU server delayed; Optimistic ~240. About 500 h in 3 months = 1 FTE (his assumption). Includes 12 h of officer training, so do not count the same training again under the trainer row.</t>
+    <t xml:space="preserve">Confirmed by Oybek (11 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-time: on-prem installation and app work. Base ~340 h (confirmed by Oybek) (his table sums to 344) = month 1: 168 (install on bank server, bank data adapter, local LLM with GPU, SSO/roles, audit to bank DB, historical test run), month 2: 96 (support, officer-feedback changes, training, monitoring), month 3: 80 (result report, documents). Pessimistic ~520 = complex data connection, many security requirements, GPU server delayed; Optimistic ~240. About 500 h in 3 months = 1 FTE (his assumption). Includes 12 h of officer training, so do not count the same training again under the trainer row.</t>
   </si>
   <si>
     <t xml:space="preserve">Pilot hours: Trainer / business analyst</t>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Calculated from official price, measured tokens (n=3)</t>
   </si>
   <si>
-    <t xml:space="preserve">Pessimistic = earlier stress value (higher-priced model, GPT-4o public price, 1,000+1,000 tokens = USD 0.0125). Base = Gemini 3.6 Flash at the 2027 price with measured tokens (~1,230 in / ~670 out, production logs, n=3) = USD 0.0069; Optimistic = the same at the 2026 price = USD 0.0034. The prototype actually runs on the free tier (USD 0 spent). Production would use a local LLM on the bank server, so this API price is only the prototype/benchmark cost. Row 58 holds the logged cost for reference only.</t>
+    <t xml:space="preserve">Pessimistic = earlier stress value (higher-priced model, GPT-4o public price, 1,000+1,000 tokens = USD 0.0125). Base = Gemini 3.6 Flash at the 2027 price with measured tokens (~1,230 in / ~670 out, production logs, n=3) = USD 0.0069; Optimistic = the same at the 2026 price = USD 0.0034. The prototype actually runs on the free tier (USD 0 spent). Production would use a local LLM on the bank server, so this API price is only the prototype/benchmark cost. Row 58 holds the logged cost for reference only. Counted in the ROI only for infrastructure options 2-3 (external API); option 1 uses a local LLM, so its API cost is 0.</t>
   </si>
   <si>
     <t xml:space="preserve">Exchange rate: 1 USD = ? UZS</t>
@@ -549,10 +549,10 @@
     <t xml:space="preserve">USD/month</t>
   </si>
   <si>
-    <t xml:space="preserve">Plan fee verified (Railway docs); actual bill not seen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD 5/month = Hobby plan fee, confirmed on docs.railway.com/pricing/plans (11 Oct 2026). Per that page the Hobby plan includes USD 5 of usage and any usage above it is billed on top, so the monthly bill is max(5, usage). The modelled usage (about 1.4 GB memory = about USD 14/month) would give a higher bill than USD 5; the actual invoice was not seen. Reference only, does not affect results.</t>
+    <t xml:space="preserve">Plan fee verified; usage screenshots pending (Oybek)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD 5/month = Hobby plan fee, confirmed on docs.railway.com/pricing/plans (11 Oct 2026). Per that page the Hobby plan includes USD 5 of usage and any usage above it is billed on top, so the monthly bill is max(5, usage). The modelled usage (about 1.4 GB memory = about USD 14/month) would give a higher bill than USD 5; the actual invoice was not seen. Reference only, does not affect results. Oybek (11 Oct): $5 is only the minimum subscription; the modelled ~USD 14/month memory usage may be closer to reality. Update this row when the Usage and Metrics screenshots arrive.</t>
   </si>
   <si>
     <t xml:space="preserve">ROI calculation (annual, UZS)</t>
@@ -663,10 +663,10 @@
     <t xml:space="preserve">N x check frequency</t>
   </si>
   <si>
-    <t xml:space="preserve">Annual LLM cost (UZS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checks x USD price per report (Assumptions row 29: measured tokens x Gemini price) x exchange rate</t>
+    <t xml:space="preserve">Annual LLM API cost, selected option (UZS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infra row 46: 0 for option 1 (local LLM, no API cost); for options 2-3 the external API price (Assumptions row 29, measured tokens x Gemini price)</t>
   </si>
   <si>
     <t xml:space="preserve">Total annual recurring cost (UZS)</t>
@@ -876,6 +876,12 @@
     <t xml:space="preserve">Total hours of the two roles over 3 months.</t>
   </si>
   <si>
+    <t xml:space="preserve">Break-even: highest share of visits still performed at which the pilot pays back within 12 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 - (annual recurring + one-time cost) / (all scheduled visits x cost per visit). Compare with the share of visits kept in each scenario (Assumptions row 9); see Sensitivity table 3.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Infrastructure cost options (measured CPU, cost.md)</t>
   </si>
   <si>
@@ -978,24 +984,27 @@
     <t xml:space="preserve">  Annual recurring cost incl. LLM (UZS)</t>
   </si>
   <si>
+    <t xml:space="preserve">Support + licences/security + hosting (0) + LLM API (0: local LLM, option 1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Annual net benefit, visit savings only (UZS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A - annual recurring cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Hardware-only payback, months (lower bound)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excludes pilot people cost (hours not entered yet).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 2: dedicated CPU server (rental)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Support + licences/security + hosting + LLM.</t>
   </si>
   <si>
-    <t xml:space="preserve">  Annual net benefit, visit savings only (UZS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A - annual recurring cost.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Hardware-only payback, months (lower bound)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excludes pilot people cost (hours not entered yet).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Option 2: dedicated CPU server (rental)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Option 3: cloud CPU (Railway)</t>
   </si>
   <si>
@@ -1023,6 +1032,21 @@
     <t xml:space="preserve">If large, check the Railway Usage page: the plan fee alone may not be the full bill.</t>
   </si>
   <si>
+    <t xml:space="preserve">E. LLM running cost by option</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual LLM API cost if an external API is used (UZS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remote checks x USD per report x exchange rate. Prototype / benchmark price (Gemini 3.6 Flash).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM API cost counted in the selected option (UZS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option 1 = local LLM on the bank server: no API cost; the GPU server (row 19) is the cost, its power and operation are not included. Options 2-3 have no GPU, so an external API is assumed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sensitivity (Base case, UZS million)</t>
   </si>
   <si>
@@ -1035,7 +1059,7 @@
     <t xml:space="preserve">visits/year \ UZS per visit</t>
   </si>
   <si>
-    <t xml:space="preserve">Grid points: 100k and 300k and 2-4 visits are the assumed range (Taxmin, unverified); 150k and 250k are interpolation; 50k is a stress case below that range. Recurring cost follows the selected infrastructure option and scales its LLM part with visits.</t>
+    <t xml:space="preserve">Grid points: 100k and 300k and 2-4 visits are the assumed range (Taxmin, unverified); 150k and 250k are interpolation; 50k is a stress case below that range. Recurring cost follows the selected infrastructure option and adds an LLM API part (options 2-3 only) that scales with visits.</t>
   </si>
   <si>
     <t xml:space="preserve">Table 2. Loss benefit vs simple rule (UZS mln): share of misused loans (rows) x share of amount recovered (columns); Base recall, N from Assumptions</t>
@@ -1149,7 +1173,7 @@
     <t xml:space="preserve">Deck summary (all values are formulas from the ROI sheet; one-branch pilot)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lead with the PESSIMISTIC column on the slide. Every input is an assumption marked 'Taxmin' unless stated.</t>
+    <t xml:space="preserve">Every input is an assumption marked 'Taxmin' unless stated.</t>
   </si>
   <si>
     <t xml:space="preserve">Loans monitored in the pilot branch</t>
@@ -1419,16 +1443,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="84">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1444,15 +1468,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1488,7 +1512,7 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1496,11 +1520,11 @@
       <alignment horizontal="right" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1560,7 +1584,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1572,7 +1596,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1652,6 +1676,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1676,7 +1704,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1700,10 +1728,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1720,15 +1744,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2017,7 +2033,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H71"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="48"/>
@@ -3564,8 +3580,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F66"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56"/>
@@ -3952,17 +3968,17 @@
       <c r="B24" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="C24" s="40" t="n">
-        <f aca="false">C23*Assumptions!C29*Assumptions!C30</f>
-        <v>456092.945</v>
-      </c>
-      <c r="D24" s="40" t="n">
-        <f aca="false">D23*Assumptions!D29*Assumptions!D30</f>
-        <v>376003.023858</v>
-      </c>
-      <c r="E24" s="40" t="n">
-        <f aca="false">E23*Assumptions!E29*Assumptions!E30</f>
-        <v>250668.682572</v>
+      <c r="C24" s="39" t="n">
+        <f aca="false">Infra!C46</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="39" t="n">
+        <f aca="false">Infra!D46</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="39" t="n">
+        <f aca="false">Infra!E46</f>
+        <v>0</v>
       </c>
       <c r="F24" s="9" t="s">
         <v>213</v>
@@ -3974,15 +3990,15 @@
       </c>
       <c r="C25" s="42" t="n">
         <f aca="false">C22+C24</f>
-        <v>73056092.945</v>
+        <v>72600000</v>
       </c>
       <c r="D25" s="42" t="n">
         <f aca="false">D22+D24</f>
-        <v>70476003.023858</v>
+        <v>70100000</v>
       </c>
       <c r="E25" s="42" t="n">
         <f aca="false">E22+E24</f>
-        <v>67850668.682572</v>
+        <v>67600000</v>
       </c>
       <c r="F25" s="9"/>
     </row>
@@ -4001,15 +4017,15 @@
       </c>
       <c r="C27" s="42" t="n">
         <f aca="false">IF(C23=0,"not entered",C25/C23)</f>
-        <v>23719.5106964286</v>
+        <v>23571.4285714286</v>
       </c>
       <c r="D27" s="42" t="n">
         <f aca="false">IF(D23=0,"not entered",D25/D23)</f>
-        <v>15254.5461090602</v>
+        <v>15173.1601731602</v>
       </c>
       <c r="E27" s="42" t="n">
         <f aca="false">IF(E23=0,"not entered",E25/E23)</f>
-        <v>11014.718941976</v>
+        <v>10974.025974026</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>217</v>
@@ -4050,15 +4066,15 @@
       </c>
       <c r="C30" s="42" t="n">
         <f aca="false">C11-C25</f>
-        <v>80943907.055</v>
+        <v>81400000</v>
       </c>
       <c r="D30" s="42" t="n">
         <f aca="false">D11-D25</f>
-        <v>668723996.976142</v>
+        <v>669100000</v>
       </c>
       <c r="E30" s="42" t="n">
         <f aca="false">E11-E25</f>
-        <v>1410549331.31743</v>
+        <v>1410800000</v>
       </c>
       <c r="F30" s="9" t="s">
         <v>222</v>
@@ -4090,15 +4106,15 @@
       </c>
       <c r="C32" s="44" t="n">
         <f aca="false">IF(C21="not entered","not entered",IF(C30&lt;=0,"no payback",C21/(C30/12)))</f>
-        <v>33.6232843091046</v>
+        <v>33.4348894348894</v>
       </c>
       <c r="D32" s="44" t="n">
         <f aca="false">IF(D21="not entered","not entered",IF(D30&lt;=0,"no payback",D21/(D30/12)))</f>
-        <v>3.14210348290367</v>
+        <v>3.1403377671499</v>
       </c>
       <c r="E32" s="44" t="n">
         <f aca="false">IF(E21="not entered","not entered",IF(E30&lt;=0,"no payback",E21/(E30/12)))</f>
-        <v>1.12977261030042</v>
+        <v>1.12957187411398</v>
       </c>
       <c r="F32" s="9" t="s">
         <v>226</v>
@@ -4159,15 +4175,15 @@
       </c>
       <c r="C37" s="47" t="n">
         <f aca="false">IF(ISNUMBER(C27),C36/C27,"not entered")</f>
-        <v>1.79598438515629E-006</v>
+        <v>1.80726724751717E-006</v>
       </c>
       <c r="D37" s="47" t="n">
         <f aca="false">IF(ISNUMBER(D27),D36/D27,"not entered")</f>
-        <v>2.79260166312204E-006</v>
+        <v>2.80758064557232E-006</v>
       </c>
       <c r="E37" s="47" t="n">
         <f aca="false">IF(ISNUMBER(E27),E36/E27,"not entered")</f>
-        <v>3.86754043010481E-006</v>
+        <v>3.88188172099842E-006</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>232</v>
@@ -4179,15 +4195,15 @@
       </c>
       <c r="C38" s="48" t="n">
         <f aca="false">IF(ISNUMBER(C27),C10/C27,"not entered")</f>
-        <v>4.21593856972172</v>
+        <v>4.24242424242424</v>
       </c>
       <c r="D38" s="48" t="n">
         <f aca="false">IF(ISNUMBER(D27),D10/D27,"not entered")</f>
-        <v>13.1108456829937</v>
+        <v>13.1811697574893</v>
       </c>
       <c r="E38" s="48" t="n">
         <f aca="false">IF(ISNUMBER(E27),E10/E27,"not entered")</f>
-        <v>27.2362827939922</v>
+        <v>27.3372781065089</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>234</v>
@@ -4208,15 +4224,15 @@
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">IF(C9=0,"n/a",C25/C9)</f>
-        <v>47439.0213928571</v>
+        <v>47142.8571428571</v>
       </c>
       <c r="D40" s="49" t="n">
         <f aca="false">IF(D9=0,"n/a",D25/D9)</f>
-        <v>19068.1826363252</v>
+        <v>18966.4502164502</v>
       </c>
       <c r="E40" s="49" t="n">
         <f aca="false">IF(E9=0,"n/a",E25/E9)</f>
-        <v>13768.39867747</v>
+        <v>13717.5324675325</v>
       </c>
       <c r="F40" s="9" t="s">
         <v>237</v>
@@ -4228,15 +4244,15 @@
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">IF(C10=0,"n/a",C25/C10)</f>
-        <v>730.56092945</v>
+        <v>726</v>
       </c>
       <c r="D41" s="49" t="n">
         <f aca="false">IF(D10=0,"n/a",D25/D10)</f>
-        <v>352.38001511929</v>
+        <v>350.5</v>
       </c>
       <c r="E41" s="49" t="n">
         <f aca="false">IF(E10=0,"n/a",E25/E10)</f>
-        <v>226.168895608573</v>
+        <v>225.333333333333</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>239</v>
@@ -4248,15 +4264,15 @@
       </c>
       <c r="C42" s="48" t="n">
         <f aca="false">IF(ISNUMBER(C40),C10/C40,"n/a")</f>
-        <v>2.10796928486086</v>
+        <v>2.12121212121212</v>
       </c>
       <c r="D42" s="48" t="n">
         <f aca="false">IF(ISNUMBER(D40),D10/D40,"n/a")</f>
-        <v>10.488676546395</v>
+        <v>10.5449358059914</v>
       </c>
       <c r="E42" s="48" t="n">
         <f aca="false">IF(ISNUMBER(E40),E10/E40,"n/a")</f>
-        <v>21.7890262351937</v>
+        <v>21.8698224852071</v>
       </c>
       <c r="F42" s="9" t="s">
         <v>241</v>
@@ -4268,15 +4284,15 @@
       </c>
       <c r="C43" s="50" t="n">
         <f aca="false">C30-C19</f>
-        <v>-61056092.945</v>
+        <v>-60600000</v>
       </c>
       <c r="D43" s="50" t="n">
         <f aca="false">D30-D19</f>
-        <v>550223996.976142</v>
+        <v>550600000</v>
       </c>
       <c r="E43" s="50" t="n">
         <f aca="false">E30-E19</f>
-        <v>1315549331.31743</v>
+        <v>1315800000</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>243</v>
@@ -4292,11 +4308,11 @@
       </c>
       <c r="D44" s="49" t="n">
         <f aca="false">IF(D43&lt;=0,0,D43/AVERAGE(Assumptions!D20:D22))</f>
-        <v>7176.83474316707</v>
+        <v>7181.73913043478</v>
       </c>
       <c r="E44" s="49" t="n">
         <f aca="false">IF(E43&lt;=0,0,E43/AVERAGE(Assumptions!E20:E22))</f>
-        <v>17159.3391041404</v>
+        <v>17162.6086956522</v>
       </c>
       <c r="F44" s="9" t="s">
         <v>245</v>
@@ -4308,15 +4324,15 @@
       </c>
       <c r="C45" s="51" t="n">
         <f aca="false">IF(C30&lt;=0,"no payback",C19/(C30/12))</f>
-        <v>21.0516153963529</v>
+        <v>20.9336609336609</v>
       </c>
       <c r="D45" s="51" t="n">
         <f aca="false">IF(D30&lt;=0,"no payback",D19/(D30/12))</f>
-        <v>2.12643782252476</v>
+        <v>2.12524286354805</v>
       </c>
       <c r="E45" s="51" t="n">
         <f aca="false">IF(E30&lt;=0,"no payback",E19/(E30/12))</f>
-        <v>0.808195767910691</v>
+        <v>0.808052168982138</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>247</v>
@@ -4517,15 +4533,15 @@
       </c>
       <c r="C56" s="54" t="n">
         <f aca="false">IFERROR(C25/(Assumptions!C6*Assumptions!C14*MAX(Assumptions!C15-C47,0)*Assumptions!C16),"n/a")</f>
-        <v>0.00384158957897586</v>
+        <v>0.00381760633768926</v>
       </c>
       <c r="D56" s="54" t="n">
         <f aca="false">IFERROR(D25/(Assumptions!D6*Assumptions!D14*MAX(Assumptions!D15-D47,0)*Assumptions!D16),"n/a")</f>
-        <v>0.00331198169922277</v>
+        <v>0.00329431164018936</v>
       </c>
       <c r="E56" s="54" t="n">
         <f aca="false">IFERROR(E25/(Assumptions!E6*Assumptions!E14*MAX(Assumptions!E15-E47,0)*Assumptions!E16),"n/a")</f>
-        <v>0.00290288818837655</v>
+        <v>0.00289216370810299</v>
       </c>
       <c r="F56" s="9" t="s">
         <v>268</v>
@@ -4537,15 +4553,15 @@
       </c>
       <c r="C57" s="55" t="n">
         <f aca="false">IFERROR(C25/(C13*Assumptions!C14*MAX(Assumptions!C15-C47,0)),"n/a")</f>
-        <v>0.128052985965862</v>
+        <v>0.127253544589642</v>
       </c>
       <c r="D57" s="55" t="n">
         <f aca="false">IFERROR(D25/(D13*Assumptions!D14*MAX(Assumptions!D15-D47,0)),"n/a")</f>
-        <v>0.0662396339844554</v>
+        <v>0.0658862328037872</v>
       </c>
       <c r="E57" s="55" t="n">
         <f aca="false">IFERROR(E25/(E13*Assumptions!E14*MAX(Assumptions!E15-E47,0)),"n/a")</f>
-        <v>0.0414698312625221</v>
+        <v>0.0413166244014712</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>270</v>
@@ -4635,15 +4651,15 @@
       </c>
       <c r="C64" s="51" t="n">
         <f aca="false">IF(NOT(ISNUMBER(C63)),"not entered",IF(C30&lt;=0,"no payback",C63/(C30/12)))</f>
-        <v>31.4884726069392</v>
+        <v>31.3120393120393</v>
       </c>
       <c r="D64" s="51" t="n">
         <f aca="false">IF(NOT(ISNUMBER(D63)),"not entered",IF(D30&lt;=0,"no payback",D63/(D30/12)))</f>
-        <v>2.9698351023447</v>
+        <v>2.96816619339411</v>
       </c>
       <c r="E64" s="51" t="n">
         <f aca="false">IF(NOT(ISNUMBER(E63)),"not entered",IF(E30&lt;=0,"no payback",E63/(E30/12)))</f>
-        <v>1.07872866706395</v>
+        <v>1.07853700028353</v>
       </c>
       <c r="F64" s="9" t="s">
         <v>280</v>
@@ -4667,6 +4683,26 @@
       </c>
       <c r="F65" s="9" t="s">
         <v>282</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="C66" s="58" t="n">
+        <f aca="false">IF(ISNUMBER(C21),1-(C25+C21)/(C7*C10),"not entered")</f>
+        <v>0.0279220779220779</v>
+      </c>
+      <c r="D66" s="58" t="n">
+        <f aca="false">IF(ISNUMBER(D21),1-(D25+D21)/(D7*D10),"not entered")</f>
+        <v>0.734632034632035</v>
+      </c>
+      <c r="E66" s="58" t="n">
+        <f aca="false">IF(ISNUMBER(E21),1-(E25+E21)/(E7*E10),"not entered")</f>
+        <v>0.891558441558442</v>
+      </c>
+      <c r="F66" s="9" t="s">
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -4688,8 +4724,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:F42"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:F46"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56"/>
@@ -4698,13 +4734,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="58" t="s">
-        <v>283</v>
+      <c r="B1" s="59" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="57" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C2" s="57"/>
       <c r="D2" s="57"/>
@@ -4712,25 +4748,25 @@
       <c r="F2" s="57"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="60" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="59" t="s">
+      <c r="C4" s="60" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="59" t="s">
+      <c r="D4" s="60" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="59" t="s">
+      <c r="E4" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="59" t="s">
+      <c r="F4" s="60" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="45" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
@@ -4739,7 +4775,7 @@
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C6" s="25" t="n">
         <f aca="false">Assumptions!C50+Assumptions!C51+Assumptions!C52</f>
@@ -4754,92 +4790,92 @@
         <v>0.466</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="C7" s="60" t="n">
+        <v>290</v>
+      </c>
+      <c r="C7" s="61" t="n">
         <f aca="false">C6*Assumptions!C54/60</f>
         <v>3.59596666666667E-006</v>
       </c>
-      <c r="D7" s="60" t="n">
+      <c r="D7" s="61" t="n">
         <f aca="false">D6*Assumptions!D54/60</f>
         <v>3.59596666666667E-006</v>
       </c>
-      <c r="E7" s="60" t="n">
+      <c r="E7" s="61" t="n">
         <f aca="false">E6*Assumptions!E54/60</f>
         <v>3.59596666666667E-006</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="C8" s="61" t="n">
+        <v>292</v>
+      </c>
+      <c r="C8" s="62" t="n">
         <f aca="false">C7*Assumptions!C30</f>
         <v>0.0425998708343333</v>
       </c>
-      <c r="D8" s="61" t="n">
+      <c r="D8" s="62" t="n">
         <f aca="false">D7*Assumptions!D30</f>
         <v>0.0425998708343333</v>
       </c>
-      <c r="E8" s="61" t="n">
+      <c r="E8" s="62" t="n">
         <f aca="false">E7*Assumptions!E30</f>
         <v>0.0425998708343333</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="C9" s="62" t="n">
+      <c r="C9" s="63" t="n">
         <f aca="false">ROI!C23</f>
         <v>3080</v>
       </c>
-      <c r="D9" s="62" t="n">
+      <c r="D9" s="63" t="n">
         <f aca="false">ROI!D23</f>
         <v>4620</v>
       </c>
-      <c r="E9" s="62" t="n">
+      <c r="E9" s="63" t="n">
         <f aca="false">ROI!E23</f>
         <v>6160</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="C10" s="61" t="n">
+        <v>295</v>
+      </c>
+      <c r="C10" s="62" t="n">
         <f aca="false">C9*C8</f>
         <v>131.207602169747</v>
       </c>
-      <c r="D10" s="61" t="n">
+      <c r="D10" s="62" t="n">
         <f aca="false">D9*D8</f>
         <v>196.81140325462</v>
       </c>
-      <c r="E10" s="61" t="n">
+      <c r="E10" s="62" t="n">
         <f aca="false">E9*E8</f>
         <v>262.415204339493</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="9" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C11" s="31" t="n">
         <f aca="false">Assumptions!C53/1024*Assumptions!C55</f>
@@ -4854,12 +4890,12 @@
         <v>13.935546875</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="C12" s="49" t="n">
         <f aca="false">C11*12*Assumptions!C30</f>
@@ -4874,12 +4910,12 @@
         <v>1981061.17851563</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="41" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C13" s="50" t="n">
         <f aca="false">C10+C12</f>
@@ -4894,12 +4930,12 @@
         <v>1981323.59371996</v>
       </c>
       <c r="F13" s="9" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="45" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -4908,7 +4944,7 @@
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B15" s="41" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C15" s="50" t="n">
         <f aca="false">12*Assumptions!C56*Assumptions!C57</f>
@@ -4923,12 +4959,12 @@
         <v>10834771.8348</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="C16" s="56" t="str">
         <f aca="false">IF(OR(Assumptions!C56="",Assumptions!C57=""),"input missing","ok")</f>
@@ -4943,12 +4979,12 @@
         <v>ok</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="45" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
@@ -4957,27 +4993,27 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="C18" s="63" t="n">
+        <v>309</v>
+      </c>
+      <c r="C18" s="64" t="n">
         <f aca="false">Assumptions!$C$49</f>
         <v>1</v>
       </c>
-      <c r="D18" s="63" t="n">
+      <c r="D18" s="64" t="n">
         <f aca="false">Assumptions!$C$49</f>
         <v>1</v>
       </c>
-      <c r="E18" s="63" t="n">
+      <c r="E18" s="64" t="n">
         <f aca="false">Assumptions!$C$49</f>
         <v>1</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C19" s="49" t="n">
         <f aca="false">CHOOSE(C18,Assumptions!C26,0,0)</f>
@@ -4992,12 +5028,12 @@
         <v>95000000</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C20" s="49" t="n">
         <f aca="false">CHOOSE(C18,0,C15,C13)</f>
@@ -5012,12 +5048,12 @@
         <v>0</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="45" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -5026,7 +5062,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="41" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
@@ -5035,7 +5071,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C23" s="49" t="n">
         <f aca="false">Assumptions!C26</f>
@@ -5053,67 +5089,67 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C24" s="49" t="n">
-        <f aca="false">Assumptions!C27+Assumptions!C28+0+ROI!C24</f>
-        <v>73056092.945</v>
+        <f aca="false">Assumptions!C27+Assumptions!C28+0+0</f>
+        <v>72600000</v>
       </c>
       <c r="D24" s="49" t="n">
-        <f aca="false">Assumptions!D27+Assumptions!D28+0+ROI!D24</f>
-        <v>70476003.023858</v>
+        <f aca="false">Assumptions!D27+Assumptions!D28+0+0</f>
+        <v>70100000</v>
       </c>
       <c r="E24" s="49" t="n">
-        <f aca="false">Assumptions!E27+Assumptions!E28+0+ROI!E24</f>
-        <v>67850668.682572</v>
+        <f aca="false">Assumptions!E27+Assumptions!E28+0+0</f>
+        <v>67600000</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C25" s="49" t="n">
         <f aca="false">ROI!C11-C24</f>
-        <v>80943907.055</v>
+        <v>81400000</v>
       </c>
       <c r="D25" s="49" t="n">
         <f aca="false">ROI!D11-D24</f>
-        <v>668723996.976142</v>
+        <v>669100000</v>
       </c>
       <c r="E25" s="49" t="n">
         <f aca="false">ROI!E11-E24</f>
-        <v>1410549331.31743</v>
+        <v>1410800000</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C26" s="53" t="n">
         <f aca="false">IF(C25&lt;=0,"no payback",C23/(C25/12))</f>
-        <v>21.0516153963529</v>
+        <v>20.9336609336609</v>
       </c>
       <c r="D26" s="53" t="n">
         <f aca="false">IF(D25&lt;=0,"no payback",D23/(D25/12))</f>
-        <v>2.12643782252476</v>
+        <v>2.12524286354805</v>
       </c>
       <c r="E26" s="53" t="n">
         <f aca="false">IF(E25&lt;=0,"no payback",E23/(E25/12))</f>
-        <v>0.808195767910691</v>
+        <v>0.808052168982138</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="41" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
@@ -5122,7 +5158,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C28" s="49" t="n">
         <f aca="false">0</f>
@@ -5140,27 +5176,27 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C29" s="49" t="n">
-        <f aca="false">Assumptions!C27+Assumptions!C28+C15+ROI!C24</f>
+        <f aca="false">Assumptions!C27+Assumptions!C28+C15+C45</f>
         <v>83890864.7798</v>
       </c>
       <c r="D29" s="49" t="n">
-        <f aca="false">Assumptions!D27+Assumptions!D28+D15+ROI!D24</f>
+        <f aca="false">Assumptions!D27+Assumptions!D28+D15+D45</f>
         <v>81310774.858658</v>
       </c>
       <c r="E29" s="49" t="n">
-        <f aca="false">Assumptions!E27+Assumptions!E28+E15+ROI!E24</f>
+        <f aca="false">Assumptions!E27+Assumptions!E28+E15+E45</f>
         <v>78685440.517372</v>
       </c>
       <c r="F29" s="9" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C30" s="49" t="n">
         <f aca="false">ROI!C11-C29</f>
@@ -5175,12 +5211,12 @@
         <v>1399714559.48263</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C31" s="53" t="n">
         <f aca="false">IF(C30&lt;=0,"no payback",C28/(C30/12))</f>
@@ -5195,12 +5231,12 @@
         <v>0</v>
       </c>
       <c r="F31" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="41" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
@@ -5209,7 +5245,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C33" s="49" t="n">
         <f aca="false">0</f>
@@ -5227,27 +5263,27 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="9" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C34" s="49" t="n">
-        <f aca="false">Assumptions!C27+Assumptions!C28+C13+ROI!C24</f>
+        <f aca="false">Assumptions!C27+Assumptions!C28+C13+C45</f>
         <v>75037285.3311178</v>
       </c>
       <c r="D34" s="49" t="n">
-        <f aca="false">Assumptions!D27+Assumptions!D28+D13+ROI!D24</f>
+        <f aca="false">Assumptions!D27+Assumptions!D28+D13+D45</f>
         <v>72457261.0137769</v>
       </c>
       <c r="E34" s="49" t="n">
-        <f aca="false">Assumptions!E27+Assumptions!E28+E13+ROI!E24</f>
+        <f aca="false">Assumptions!E27+Assumptions!E28+E13+E45</f>
         <v>69831992.276292</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C35" s="49" t="n">
         <f aca="false">ROI!C11-C34</f>
@@ -5262,12 +5298,12 @@
         <v>1408568007.72371</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="9" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C36" s="53" t="n">
         <f aca="false">IF(C35&lt;=0,"no payback",C33/(C35/12))</f>
@@ -5282,12 +5318,12 @@
         <v>0</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="57" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C37" s="57"/>
       <c r="D37" s="57"/>
@@ -5295,13 +5331,13 @@
       <c r="F37" s="57"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="64" t="s">
-        <v>325</v>
+      <c r="B39" s="65" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="9" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C40" s="49" t="n">
         <f aca="false">Assumptions!C71*12*Assumptions!C30</f>
@@ -5316,12 +5352,12 @@
         <v>710794.2</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="9" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="C41" s="49" t="n">
         <f aca="false">C13</f>
@@ -5336,12 +5372,12 @@
         <v>1981323.59371996</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="9" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="C42" s="49" t="n">
         <f aca="false">C41-C40</f>
@@ -5356,7 +5392,56 @@
         <v>1270529.39371996</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>331</v>
+        <v>334</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="C44" s="35"/>
+      <c r="D44" s="35"/>
+      <c r="E44" s="35"/>
+      <c r="F44" s="35"/>
+    </row>
+    <row r="45" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="C45" s="49" t="n">
+        <f aca="false">ROI!C23*Assumptions!C29*Assumptions!C30</f>
+        <v>456092.945</v>
+      </c>
+      <c r="D45" s="49" t="n">
+        <f aca="false">ROI!D23*Assumptions!D29*Assumptions!D30</f>
+        <v>376003.023858</v>
+      </c>
+      <c r="E45" s="49" t="n">
+        <f aca="false">ROI!E23*Assumptions!E29*Assumptions!E30</f>
+        <v>250668.682572</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="C46" s="49" t="n">
+        <f aca="false">IF(C18=1,0,C45)</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="49" t="n">
+        <f aca="false">IF(D18=1,0,D45)</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="49" t="n">
+        <f aca="false">IF(E18=1,0,E45)</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -5380,7 +5465,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:H26"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="38"/>
@@ -5388,13 +5473,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="58" t="s">
-        <v>332</v>
+      <c r="B1" s="59" t="s">
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="57" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="C2" s="57"/>
       <c r="D2" s="57"/>
@@ -5404,129 +5489,129 @@
       <c r="H2" s="57"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="65" t="s">
-        <v>334</v>
-      </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="65"/>
-      <c r="H4" s="65"/>
+      <c r="B4" s="66" t="s">
+        <v>342</v>
+      </c>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="66" t="s">
-        <v>335</v>
-      </c>
-      <c r="C5" s="67" t="n">
+      <c r="B5" s="67" t="s">
+        <v>343</v>
+      </c>
+      <c r="C5" s="68" t="n">
         <v>50000</v>
       </c>
-      <c r="D5" s="67" t="n">
+      <c r="D5" s="68" t="n">
         <v>100000</v>
       </c>
-      <c r="E5" s="67" t="n">
+      <c r="E5" s="68" t="n">
         <v>150000</v>
       </c>
-      <c r="F5" s="67" t="n">
+      <c r="F5" s="68" t="n">
         <v>200000</v>
       </c>
-      <c r="G5" s="67" t="n">
+      <c r="G5" s="68" t="n">
         <v>250000</v>
       </c>
-      <c r="H5" s="67" t="n">
+      <c r="H5" s="68" t="n">
         <v>300000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="68" t="n">
+      <c r="B6" s="69" t="n">
         <v>2</v>
       </c>
       <c r="C6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>52.849331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>53.1</v>
       </c>
       <c r="D6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>176.049331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>176.3</v>
       </c>
       <c r="E6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>299.249331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>299.5</v>
       </c>
       <c r="F6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>422.449331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>422.7</v>
       </c>
       <c r="G6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>545.649331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>545.9</v>
       </c>
       <c r="H6" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>668.849331317428</v>
+        <f aca="false">(Assumptions!$D$6*$B6*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B6*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>669.1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="68" t="n">
+      <c r="B7" s="69" t="n">
         <v>3</v>
       </c>
       <c r="C7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>114.323996976142</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>114.7</v>
       </c>
       <c r="D7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>299.123996976142</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>299.5</v>
       </c>
       <c r="E7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>483.923996976142</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>484.3</v>
       </c>
       <c r="F7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>668.723996976142</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>669.1</v>
       </c>
       <c r="G7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>853.523996976142</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>853.9</v>
       </c>
       <c r="H7" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>1038.32399697614</v>
+        <f aca="false">(Assumptions!$D$6*$B7*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B7*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>1038.7</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="68" t="n">
+      <c r="B8" s="69" t="n">
         <v>4</v>
       </c>
       <c r="C8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>175.798662634856</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*C$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>176.3</v>
       </c>
       <c r="D8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>422.198662634856</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*D$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>422.7</v>
       </c>
       <c r="E8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>668.598662634856</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*E$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>669.1</v>
       </c>
       <c r="F8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>914.998662634856</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*F$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>915.5</v>
       </c>
       <c r="G8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>1161.39866263486</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*G$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>1161.9</v>
       </c>
       <c r="H8" s="53" t="n">
-        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30))/1000000</f>
-        <v>1407.79866263486</v>
+        <f aca="false">(Assumptions!$D$6*$B8*(1-Assumptions!$D$9)*H$5-(Assumptions!$D$27+Assumptions!$D$28+Infra!$D$20+Assumptions!$D$6*$B8*Assumptions!$D$29*Assumptions!$D$30*(Assumptions!$C$49&lt;&gt;1)))/1000000</f>
+        <v>1408.3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="57" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="C9" s="57"/>
       <c r="D9" s="57"/>
@@ -5536,35 +5621,35 @@
       <c r="H9" s="57"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="65" t="s">
-        <v>337</v>
-      </c>
-      <c r="C11" s="65"/>
-      <c r="D11" s="65"/>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65"/>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
+      <c r="B11" s="66" t="s">
+        <v>345</v>
+      </c>
+      <c r="C11" s="66"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="66"/>
+      <c r="G11" s="66"/>
+      <c r="H11" s="66"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="66" t="s">
-        <v>338</v>
-      </c>
-      <c r="C12" s="69" t="n">
+      <c r="B12" s="67" t="s">
+        <v>346</v>
+      </c>
+      <c r="C12" s="70" t="n">
         <v>0.25</v>
       </c>
-      <c r="D12" s="69" t="n">
+      <c r="D12" s="70" t="n">
         <v>0.5</v>
       </c>
-      <c r="E12" s="69" t="n">
+      <c r="E12" s="70" t="n">
         <v>0.75</v>
       </c>
-      <c r="F12" s="69" t="n">
+      <c r="F12" s="70" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="69" t="n">
+      <c r="B13" s="70" t="n">
         <v>0.03</v>
       </c>
       <c r="C13" s="53" t="n">
@@ -5585,7 +5670,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="69" t="n">
+      <c r="B14" s="70" t="n">
         <v>0.05</v>
       </c>
       <c r="C14" s="53" t="n">
@@ -5606,7 +5691,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="69" t="n">
+      <c r="B15" s="70" t="n">
         <v>0.07</v>
       </c>
       <c r="C15" s="53" t="n">
@@ -5627,7 +5712,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="69" t="n">
+      <c r="B16" s="70" t="n">
         <v>0.13</v>
       </c>
       <c r="C16" s="53" t="n">
@@ -5649,7 +5734,7 @@
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="57" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="C17" s="57"/>
       <c r="D17" s="57"/>
@@ -5658,90 +5743,90 @@
       <c r="G17" s="57"/>
       <c r="H17" s="57"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="70" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="65" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="71" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C20" s="71" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="D20" s="71" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="72" t="n">
         <v>0.2</v>
       </c>
       <c r="C21" s="73" t="n">
         <f aca="false">(Assumptions!$D$6*Assumptions!$D$7*(1-$B21)*Assumptions!$D$8-ROI!$D$25)/1000000</f>
-        <v>668.723996976142</v>
+        <v>669.1</v>
       </c>
       <c r="D21" s="74" t="n">
         <f aca="false">IF(ISNUMBER(ROI!$D$21),IF(C21&lt;=0,"no payback",ROI!$D$21/(C21*1000000/12)),"not entered")</f>
-        <v>3.14210348290367</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.1403377671499</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="72" t="n">
         <v>0.3</v>
       </c>
       <c r="C22" s="73" t="n">
         <f aca="false">(Assumptions!$D$6*Assumptions!$D$7*(1-$B22)*Assumptions!$D$8-ROI!$D$25)/1000000</f>
-        <v>576.323996976142</v>
+        <v>576.7</v>
       </c>
       <c r="D22" s="74" t="n">
         <f aca="false">IF(ISNUMBER(ROI!$D$21),IF(C22&lt;=0,"no payback",ROI!$D$21/(C22*1000000/12)),"not entered")</f>
-        <v>3.64586588624555</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.64348881567539</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="72" t="n">
         <v>0.4</v>
       </c>
       <c r="C23" s="73" t="n">
         <f aca="false">(Assumptions!$D$6*Assumptions!$D$7*(1-$B23)*Assumptions!$D$8-ROI!$D$25)/1000000</f>
-        <v>483.923996976142</v>
+        <v>484.3</v>
       </c>
       <c r="D23" s="74" t="n">
         <f aca="false">IF(ISNUMBER(ROI!$D$21),IF(C23&lt;=0,"no payback",ROI!$D$21/(C23*1000000/12)),"not entered")</f>
-        <v>4.34200414348039</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>4.33863307867025</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B24" s="72" t="n">
         <v>0.5</v>
       </c>
       <c r="C24" s="73" t="n">
         <f aca="false">(Assumptions!$D$6*Assumptions!$D$7*(1-$B24)*Assumptions!$D$8-ROI!$D$25)/1000000</f>
-        <v>391.523996976142</v>
+        <v>391.9</v>
       </c>
       <c r="D24" s="74" t="n">
         <f aca="false">IF(ISNUMBER(ROI!$D$21),IF(C24&lt;=0,"no payback",ROI!$D$21/(C24*1000000/12)),"not entered")</f>
-        <v>5.36672085549852</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5.36157182954835</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="72" t="n">
         <v>0.6</v>
       </c>
       <c r="C25" s="73" t="n">
         <f aca="false">(Assumptions!$D$6*Assumptions!$D$7*(1-$B25)*Assumptions!$D$8-ROI!$D$25)/1000000</f>
-        <v>299.123996976142</v>
+        <v>299.5</v>
       </c>
       <c r="D25" s="74" t="n">
         <f aca="false">IF(ISNUMBER(ROI!$D$21),IF(C25&lt;=0,"no payback",ROI!$D$21/(C25*1000000/12)),"not entered")</f>
-        <v>7.02451164480659</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="75" t="s">
-        <v>344</v>
+        <v>7.01569282136895</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="1" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -5768,7 +5853,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:F22"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="46"/>
@@ -5777,13 +5862,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B1" s="58" t="s">
-        <v>345</v>
+      <c r="B1" s="59" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B2" s="57" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="C2" s="57"/>
       <c r="D2" s="57"/>
@@ -5791,162 +5876,162 @@
       <c r="F2" s="57"/>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="66" t="s">
-        <v>347</v>
-      </c>
-      <c r="C4" s="66" t="s">
-        <v>348</v>
-      </c>
-      <c r="D4" s="66" t="s">
-        <v>349</v>
-      </c>
-      <c r="E4" s="66" t="s">
-        <v>350</v>
+      <c r="B4" s="67" t="s">
+        <v>355</v>
+      </c>
+      <c r="C4" s="67" t="s">
+        <v>356</v>
+      </c>
+      <c r="D4" s="67" t="s">
+        <v>357</v>
+      </c>
+      <c r="E4" s="67" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="9" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="D5" s="76" t="n">
+        <v>360</v>
+      </c>
+      <c r="D5" s="75" t="n">
         <v>49400000</v>
       </c>
-      <c r="E5" s="76" t="n">
+      <c r="E5" s="75" t="n">
         <v>49700000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="9" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="D6" s="76" t="n">
+        <v>360</v>
+      </c>
+      <c r="D6" s="75" t="n">
         <v>27100000</v>
       </c>
-      <c r="E6" s="76" t="n">
+      <c r="E6" s="75" t="n">
         <v>27800000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="9" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="D7" s="76" t="n">
+        <v>360</v>
+      </c>
+      <c r="D7" s="75" t="n">
         <v>58200000</v>
       </c>
-      <c r="E7" s="76" t="n">
+      <c r="E7" s="75" t="n">
         <v>58500000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="9" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="D8" s="76" t="n">
+        <v>360</v>
+      </c>
+      <c r="D8" s="75" t="n">
         <v>41900000</v>
       </c>
-      <c r="E8" s="76" t="n">
+      <c r="E8" s="75" t="n">
         <v>41300000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="9" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>352</v>
-      </c>
-      <c r="D9" s="76" t="n">
+        <v>360</v>
+      </c>
+      <c r="D9" s="75" t="n">
         <v>99400000</v>
       </c>
-      <c r="E9" s="76" t="n">
+      <c r="E9" s="75" t="n">
         <v>91200000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="9" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="D10" s="76" t="n">
+        <v>366</v>
+      </c>
+      <c r="D10" s="75" t="n">
         <v>28600000</v>
       </c>
-      <c r="E10" s="76" t="n">
+      <c r="E10" s="75" t="n">
         <v>29700000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="9" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>360</v>
-      </c>
-      <c r="D11" s="76" t="n">
+        <v>368</v>
+      </c>
+      <c r="D11" s="75" t="n">
         <v>33900000</v>
       </c>
-      <c r="E11" s="76" t="n">
+      <c r="E11" s="75" t="n">
         <v>32600000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="9" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="D12" s="76" t="n">
+        <v>370</v>
+      </c>
+      <c r="D12" s="75" t="n">
         <v>99200000</v>
       </c>
-      <c r="E12" s="76" t="n">
+      <c r="E12" s="75" t="n">
         <v>97100000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="9" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>364</v>
-      </c>
-      <c r="D13" s="76" t="n">
+        <v>372</v>
+      </c>
+      <c r="D13" s="75" t="n">
         <v>114300000</v>
       </c>
-      <c r="E13" s="76" t="n">
+      <c r="E13" s="75" t="n">
         <v>108900000</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="9" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="D14" s="76" t="n">
+        <v>366</v>
+      </c>
+      <c r="D14" s="75" t="n">
         <v>48400000</v>
       </c>
-      <c r="E14" s="76" t="n">
+      <c r="E14" s="75" t="n">
         <v>46800000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="9" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C16" s="23" t="n">
         <f aca="false">COUNTA(B5:B14)</f>
@@ -5955,7 +6040,7 @@
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B17" s="9" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="C17" s="23" t="n">
         <f aca="false">COUNTIF(C5:C14,"&lt;&gt;halol")</f>
@@ -5964,7 +6049,7 @@
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="9" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C18" s="49" t="n">
         <f aca="false">AVERAGE(D5:D14)</f>
@@ -5973,7 +6058,7 @@
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="9" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C19" s="49" t="n">
         <f aca="false">AVERAGEIF(C5:C14,"&lt;&gt;halol",D5:D14)</f>
@@ -5982,25 +6067,25 @@
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="9" t="s">
-        <v>370</v>
-      </c>
-      <c r="C20" s="62" t="n">
+        <v>378</v>
+      </c>
+      <c r="C20" s="63" t="n">
         <f aca="false">Assumptions!D14</f>
         <v>27200000</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="9" t="s">
-        <v>371</v>
-      </c>
-      <c r="C21" s="77" t="n">
+        <v>379</v>
+      </c>
+      <c r="C21" s="58" t="n">
         <f aca="false">IF(C18=0,"n/a",C20/C18)</f>
         <v>0.453031312458361</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="57" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C22" s="57"/>
       <c r="D22" s="57"/>
@@ -6028,214 +6113,214 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:E17"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="78" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="79" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="80" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1" s="76" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B2" s="77" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="78" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="80" t="s">
+      <c r="C4" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="80" t="s">
+      <c r="D4" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="80" t="s">
+      <c r="E4" s="78" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="81" t="s">
-        <v>375</v>
-      </c>
-      <c r="C5" s="82" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="79" t="s">
+        <v>383</v>
+      </c>
+      <c r="C5" s="80" t="n">
         <f aca="false">ROI!C6</f>
         <v>1540</v>
       </c>
-      <c r="D5" s="82" t="n">
+      <c r="D5" s="80" t="n">
         <f aca="false">ROI!D6</f>
         <v>1540</v>
       </c>
-      <c r="E5" s="82" t="n">
+      <c r="E5" s="80" t="n">
         <f aca="false">ROI!E6</f>
         <v>1540</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="81" t="s">
-        <v>376</v>
-      </c>
-      <c r="C6" s="82" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="79" t="s">
+        <v>384</v>
+      </c>
+      <c r="C6" s="80" t="n">
         <f aca="false">ROI!C9</f>
         <v>1540</v>
       </c>
-      <c r="D6" s="82" t="n">
+      <c r="D6" s="80" t="n">
         <f aca="false">ROI!D9</f>
         <v>3696</v>
       </c>
-      <c r="E6" s="82" t="n">
+      <c r="E6" s="80" t="n">
         <f aca="false">ROI!E9</f>
         <v>4928</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="81" t="s">
-        <v>377</v>
-      </c>
-      <c r="C7" s="83" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="79" t="s">
+        <v>385</v>
+      </c>
+      <c r="C7" s="81" t="n">
         <f aca="false">ROI!C11/1000000</f>
         <v>154</v>
       </c>
-      <c r="D7" s="83" t="n">
+      <c r="D7" s="81" t="n">
         <f aca="false">ROI!D11/1000000</f>
         <v>739.2</v>
       </c>
-      <c r="E7" s="83" t="n">
+      <c r="E7" s="81" t="n">
         <f aca="false">ROI!E11/1000000</f>
         <v>1478.4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="81" t="s">
-        <v>378</v>
-      </c>
-      <c r="C8" s="83" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B8" s="79" t="s">
+        <v>386</v>
+      </c>
+      <c r="C8" s="81" t="n">
         <f aca="false">ROI!C25/1000000</f>
-        <v>73.056092945</v>
-      </c>
-      <c r="D8" s="83" t="n">
+        <v>72.6</v>
+      </c>
+      <c r="D8" s="81" t="n">
         <f aca="false">ROI!D25/1000000</f>
-        <v>70.476003023858</v>
-      </c>
-      <c r="E8" s="83" t="n">
+        <v>70.1</v>
+      </c>
+      <c r="E8" s="81" t="n">
         <f aca="false">ROI!E25/1000000</f>
-        <v>67.850668682572</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="81" t="s">
-        <v>379</v>
-      </c>
-      <c r="C9" s="83" t="n">
+        <v>67.6</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="79" t="s">
+        <v>387</v>
+      </c>
+      <c r="C9" s="81" t="n">
         <f aca="false">ROI!C30/1000000</f>
-        <v>80.943907055</v>
-      </c>
-      <c r="D9" s="83" t="n">
+        <v>81.4</v>
+      </c>
+      <c r="D9" s="81" t="n">
         <f aca="false">ROI!D30/1000000</f>
-        <v>668.723996976142</v>
-      </c>
-      <c r="E9" s="83" t="n">
+        <v>669.1</v>
+      </c>
+      <c r="E9" s="81" t="n">
         <f aca="false">ROI!E30/1000000</f>
-        <v>1410.54933131743</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="81" t="s">
-        <v>380</v>
-      </c>
-      <c r="C10" s="83" t="n">
+        <v>1410.8</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="79" t="s">
+        <v>388</v>
+      </c>
+      <c r="C10" s="81" t="n">
         <f aca="false">IF(ISNUMBER(ROI!C21),ROI!C21/1000000,ROI!C21)</f>
         <v>226.8</v>
       </c>
-      <c r="D10" s="83" t="n">
+      <c r="D10" s="81" t="n">
         <f aca="false">IF(ISNUMBER(ROI!D21),ROI!D21/1000000,ROI!D21)</f>
         <v>175.1</v>
       </c>
-      <c r="E10" s="83" t="n">
+      <c r="E10" s="81" t="n">
         <f aca="false">IF(ISNUMBER(ROI!E21),ROI!E21/1000000,ROI!E21)</f>
         <v>132.8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="81" t="s">
-        <v>381</v>
-      </c>
-      <c r="C11" s="84" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="79" t="s">
+        <v>389</v>
+      </c>
+      <c r="C11" s="82" t="n">
         <f aca="false">ROI!C32</f>
-        <v>33.6232843091046</v>
-      </c>
-      <c r="D11" s="84" t="n">
+        <v>33.4348894348894</v>
+      </c>
+      <c r="D11" s="82" t="n">
         <f aca="false">ROI!D32</f>
-        <v>3.14210348290367</v>
-      </c>
-      <c r="E11" s="84" t="n">
+        <v>3.1403377671499</v>
+      </c>
+      <c r="E11" s="82" t="n">
         <f aca="false">ROI!E32</f>
-        <v>1.12977261030042</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="81" t="s">
-        <v>382</v>
-      </c>
-      <c r="C12" s="82" t="n">
+        <v>1.12957187411398</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B12" s="79" t="s">
+        <v>390</v>
+      </c>
+      <c r="C12" s="80" t="n">
         <f aca="false">ROI!C27</f>
-        <v>23719.5106964286</v>
-      </c>
-      <c r="D12" s="82" t="n">
+        <v>23571.4285714286</v>
+      </c>
+      <c r="D12" s="80" t="n">
         <f aca="false">ROI!D27</f>
-        <v>15254.5461090602</v>
-      </c>
-      <c r="E12" s="82" t="n">
+        <v>15173.1601731602</v>
+      </c>
+      <c r="E12" s="80" t="n">
         <f aca="false">ROI!E27</f>
-        <v>11014.718941976</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="81" t="s">
-        <v>383</v>
-      </c>
-      <c r="C13" s="82" t="n">
+        <v>10974.025974026</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B13" s="79" t="s">
+        <v>391</v>
+      </c>
+      <c r="C13" s="80" t="n">
         <f aca="false">ROI!C28</f>
         <v>100000</v>
       </c>
-      <c r="D13" s="82" t="n">
+      <c r="D13" s="80" t="n">
         <f aca="false">ROI!D28</f>
         <v>200000</v>
       </c>
-      <c r="E13" s="82" t="n">
+      <c r="E13" s="80" t="n">
         <f aca="false">ROI!E28</f>
         <v>300000</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="81" t="s">
-        <v>384</v>
-      </c>
-      <c r="C14" s="85" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B14" s="79" t="s">
+        <v>392</v>
+      </c>
+      <c r="C14" s="83" t="n">
         <f aca="false">Assumptions!C15</f>
         <v>0.728</v>
       </c>
-      <c r="D14" s="85" t="n">
+      <c r="D14" s="83" t="n">
         <f aca="false">Assumptions!D15</f>
         <v>0.782</v>
       </c>
-      <c r="E14" s="85" t="n">
+      <c r="E14" s="83" t="n">
         <f aca="false">Assumptions!E15</f>
         <v>0.832</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="79" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="79" t="s">
-        <v>386</v>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B16" s="77" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="77" t="s">
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>